<commit_message>
Updates to CAN Logger
</commit_message>
<xml_diff>
--- a/Max/Arduino/Arduino Board Testing/High Res Testing and Tuneing/Data.xlsx
+++ b/Max/Arduino/Arduino Board Testing/High Res Testing and Tuneing/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/mahf202_exeter_ac_uk/Documents/4th Year Design Project/Code/Solex/Max/Arduino/Arduino Board Testing/High Res Testing and Tuneing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="308" documentId="8_{01A00817-EADD-4DE4-AA49-850561A66BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34222533-3FCE-4518-B97A-4B54A7539142}"/>
+  <xr:revisionPtr revIDLastSave="372" documentId="8_{01A00817-EADD-4DE4-AA49-850561A66BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7394B1D4-3A41-4C28-B7EF-E91ED39E8A81}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{5D5FDD7C-948B-43F0-8236-2633AF66ED44}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{5D5FDD7C-948B-43F0-8236-2633AF66ED44}"/>
   </bookViews>
   <sheets>
     <sheet name="Battery Voltage" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,6 @@
     <sheet name="Solar Current" sheetId="3" r:id="rId3"/>
     <sheet name="Auxiliary" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'Battery Voltage'!$A$2:$A$34</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Battery Voltage'!$B$2:$B$34</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'Battery Voltage'!$C$2:$C$34</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'Battery Voltage'!$A$2:$A$34</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'Battery Voltage'!$B$2:$B$34</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'Battery Voltage'!$C$2:$C$34</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -47,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="13">
   <si>
     <t>Input</t>
   </si>
@@ -74,6 +66,18 @@
   </si>
   <si>
     <t>Measurement</t>
+  </si>
+  <si>
+    <t>[0</t>
+  </si>
+  <si>
+    <t>0.008]</t>
+  </si>
+  <si>
+    <t>0.1 0.2</t>
+  </si>
+  <si>
+    <t>]</t>
   </si>
 </sst>
 </file>
@@ -217,15 +221,6 @@
                 <c:pt idx="3">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>30</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -239,22 +234,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.88</c:v>
+                  <c:v>4.7850000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.84</c:v>
+                  <c:v>9.8000000000000007</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14.84</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>19.8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>24.8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>29.75</c:v>
+                  <c:v>14.76</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -378,15 +364,6 @@
                 <c:pt idx="3">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>30</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -400,22 +377,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.12000000000000011</c:v>
+                  <c:v>0.21499999999999986</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.16000000000000014</c:v>
+                  <c:v>0.19999999999999929</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.16000000000000014</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.19999999999999929</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.19999999999999929</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.25</c:v>
+                  <c:v>0.24000000000000021</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -475,15 +443,6 @@
                 <c:pt idx="3">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>30</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -497,22 +456,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.88</c:v>
+                  <c:v>4.7850000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.84</c:v>
+                  <c:v>9.8000000000000007</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14.84</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>19.8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>24.8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>29.75</c:v>
+                  <c:v>14.76</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -778,19 +728,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -802,19 +752,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -863,19 +813,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -887,19 +837,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8.26</c:v>
+                  <c:v>7.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.1</c:v>
+                  <c:v>10.509</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16.02</c:v>
+                  <c:v>13.846</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>19.93</c:v>
+                  <c:v>17.396000000000001</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>23.92</c:v>
+                  <c:v>20.661999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1012,19 +962,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1036,19 +986,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-0.25999999999999979</c:v>
+                  <c:v>-9.9999999999999645E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-9.9999999999999645E-2</c:v>
+                  <c:v>-9.0000000000003411E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1.9999999999999574E-2</c:v>
+                  <c:v>0.15399999999999991</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.0000000000000284E-2</c:v>
+                  <c:v>0.1039999999999992</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.9999999999998295E-2</c:v>
+                  <c:v>0.33800000000000097</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1097,19 +1047,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1121,19 +1071,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>7.07</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>10.507999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>14.012</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>17.516999999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>21.021999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1232,19 +1182,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>24</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1256,19 +1206,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>-8</c:v>
+                  <c:v>7.0000000000000284E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-12</c:v>
+                  <c:v>7.9999999999991189E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-16</c:v>
+                  <c:v>1.2000000000000455E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-20</c:v>
+                  <c:v>1.699999999999946E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-24</c:v>
+                  <c:v>2.1999999999998465E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1542,19 +1492,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.5</c:v>
+                  <c:v>5.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.5</c:v>
+                  <c:v>8.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1566,19 +1516,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.5</c:v>
+                  <c:v>5.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.5</c:v>
+                  <c:v>8.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1635,19 +1585,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.5</c:v>
+                  <c:v>5.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.5</c:v>
+                  <c:v>8.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1659,19 +1609,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9.0399999999999991</c:v>
+                  <c:v>3.621</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.52</c:v>
+                  <c:v>5.3609999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>17.79</c:v>
+                  <c:v>7.0650000000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.21</c:v>
+                  <c:v>8.7690000000000001</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>26.76</c:v>
+                  <c:v>10.36</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1778,19 +1728,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.5</c:v>
+                  <c:v>5.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.5</c:v>
+                  <c:v>8.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1802,19 +1752,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-3.9999999999999147E-2</c:v>
+                  <c:v>-0.121</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1.9999999999999574E-2</c:v>
+                  <c:v>-0.11099999999999977</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.21000000000000085</c:v>
+                  <c:v>-6.5000000000000391E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.28999999999999915</c:v>
+                  <c:v>-1.9000000000000128E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.23999999999999844</c:v>
+                  <c:v>0.14000000000000057</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1871,19 +1821,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.5</c:v>
+                  <c:v>5.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.5</c:v>
+                  <c:v>8.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1895,19 +1845,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9.07</c:v>
+                  <c:v>3.5339999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.57</c:v>
+                  <c:v>5.29</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18.07</c:v>
+                  <c:v>7.0990000000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.35</c:v>
+                  <c:v>8.7560000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>10.56</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1964,19 +1914,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13.5</c:v>
+                  <c:v>5.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22.5</c:v>
+                  <c:v>8.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>27</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1988,19 +1938,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>7.0000000000000284E-2</c:v>
+                  <c:v>3.3999999999999808E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.0000000000000284E-2</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.0000000000000284E-2</c:v>
+                  <c:v>9.9000000000000199E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.14999999999999858</c:v>
+                  <c:v>6.0000000000002274E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>6.0000000000000497E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2391,19 +2341,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>10.46</c:v>
+                  <c:v>10.29</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15.37</c:v>
+                  <c:v>14.98</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.36</c:v>
+                  <c:v>20.09</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>25.41</c:v>
+                  <c:v>24.85</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>30.25</c:v>
+                  <c:v>30.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2534,19 +2484,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-0.46000000000000085</c:v>
+                  <c:v>-0.28999999999999915</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-0.36999999999999922</c:v>
+                  <c:v>1.9999999999999574E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-0.35999999999999943</c:v>
+                  <c:v>-8.9999999999999858E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.41000000000000014</c:v>
+                  <c:v>0.14999999999999858</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-0.25</c:v>
+                  <c:v>-0.10000000000000142</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2627,19 +2577,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9.9600000000000009</c:v>
+                  <c:v>9.99</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15.02</c:v>
+                  <c:v>15.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>19.97</c:v>
+                  <c:v>20.02</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>25.03</c:v>
+                  <c:v>24.98</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>30.04</c:v>
+                  <c:v>29.93</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2720,19 +2670,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-3.9999999999999147E-2</c:v>
+                  <c:v>-9.9999999999997868E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>9.9999999999997868E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>1.9999999999999574E-2</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>-3.0000000000001137E-2</c:v>
-                </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0000000000001137E-2</c:v>
+                  <c:v>-1.9999999999999574E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.9999999999999147E-2</c:v>
+                  <c:v>-7.0000000000000284E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5200,16 +5150,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>491260</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>568726</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>361991</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>165287</xdr:rowOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>124842</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5644,7 +5594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F953CB46-9921-46F4-91A7-446FFE25AD64}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:X61"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.46484375" bestFit="1" customWidth="1"/>
@@ -5654,7 +5604,7 @@
     <col min="5" max="5" width="5.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -5671,7 +5621,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
@@ -5689,16 +5639,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>5</v>
       </c>
       <c r="B3">
-        <v>4.88</v>
+        <v>4.7850000000000001</v>
       </c>
       <c r="C3">
         <f t="shared" ref="C3:C8" si="0">A3-B3</f>
-        <v>0.12000000000000011</v>
+        <v>0.21499999999999986</v>
       </c>
       <c r="D3">
         <v>4.97</v>
@@ -5708,99 +5658,372 @@
         <v>3.0000000000000249E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>10</v>
       </c>
       <c r="B4">
-        <v>9.84</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>0.16000000000000014</v>
+        <v>0.19999999999999929</v>
       </c>
       <c r="D4">
-        <v>9.9600000000000009</v>
+        <v>10.01</v>
       </c>
       <c r="E4">
         <f t="shared" ref="E4:E8" si="1">A4-D4</f>
-        <v>3.9999999999999147E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+        <v>-9.9999999999997868E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>15</v>
       </c>
       <c r="B5">
-        <v>14.84</v>
+        <v>14.76</v>
       </c>
       <c r="C5">
         <f t="shared" si="0"/>
-        <v>0.16000000000000014</v>
+        <v>0.24000000000000021</v>
       </c>
       <c r="D5">
-        <v>14.97</v>
+        <v>15.106</v>
       </c>
       <c r="E5">
         <f t="shared" si="1"/>
-        <v>2.9999999999999361E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A6">
-        <v>20</v>
-      </c>
-      <c r="B6">
-        <v>19.8</v>
-      </c>
-      <c r="C6">
-        <f t="shared" si="0"/>
-        <v>0.19999999999999929</v>
-      </c>
-      <c r="D6">
-        <v>19.98</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
-        <v>1.9999999999999574E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A7">
-        <v>25</v>
-      </c>
-      <c r="B7">
-        <v>24.8</v>
-      </c>
-      <c r="C7">
-        <f t="shared" si="0"/>
-        <v>0.19999999999999929</v>
-      </c>
-      <c r="D7">
-        <v>25.01</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="1"/>
-        <v>-1.0000000000001563E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A8">
-        <v>30</v>
-      </c>
-      <c r="B8">
-        <v>29.75</v>
-      </c>
-      <c r="C8">
-        <f t="shared" si="0"/>
-        <v>0.25</v>
-      </c>
-      <c r="D8">
-        <v>30.01</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="1"/>
-        <v>-1.0000000000001563E-2</v>
+        <v>-0.10599999999999987</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="W16" t="s">
+        <v>9</v>
+      </c>
+      <c r="X16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W17">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="X17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W18">
+        <v>1.6E-2</v>
+      </c>
+      <c r="X18">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="19" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W19">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="X19">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="20" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W20">
+        <v>2.4E-2</v>
+      </c>
+      <c r="X20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W21">
+        <v>0.03</v>
+      </c>
+      <c r="X21">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="22" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W22">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="X22">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="23" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W23">
+        <v>0.06</v>
+      </c>
+      <c r="X23">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="24" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W24">
+        <v>0.1</v>
+      </c>
+      <c r="X24">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="25" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W25">
+        <v>0.15</v>
+      </c>
+      <c r="X25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W26">
+        <v>0.18</v>
+      </c>
+      <c r="X26">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W27">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="X27">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="28" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W28">
+        <v>0.214</v>
+      </c>
+      <c r="X28">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="29" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W29">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="X29">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="30" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W30">
+        <v>0.22</v>
+      </c>
+      <c r="X30">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="31" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W31">
+        <v>0.19</v>
+      </c>
+      <c r="X31">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="32" spans="23:24" x14ac:dyDescent="0.45">
+      <c r="W32">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="X32">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="33" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="W33">
+        <v>0.12</v>
+      </c>
+      <c r="X33">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="34" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="W34">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="X34">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="35" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="W35" t="s">
+        <v>10</v>
+      </c>
+      <c r="X35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="X36" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L42">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="M42" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L43">
+        <v>1.6E-2</v>
+      </c>
+      <c r="M43">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="44" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L44">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="M44">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="45" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L45">
+        <v>2.4E-2</v>
+      </c>
+      <c r="M45">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="46" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L46">
+        <v>0.03</v>
+      </c>
+      <c r="M46">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="47" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L47">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="M47">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="48" spans="12:24" x14ac:dyDescent="0.45">
+      <c r="L48">
+        <v>0.06</v>
+      </c>
+      <c r="M48">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="49" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L49">
+        <v>0.1</v>
+      </c>
+      <c r="M49">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="50" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L50">
+        <v>0.15</v>
+      </c>
+      <c r="M50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L51">
+        <v>0.18</v>
+      </c>
+      <c r="M51">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L52">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="M52">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="53" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L53">
+        <v>0.214</v>
+      </c>
+      <c r="M53">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="54" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L54">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="M54">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="55" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L55">
+        <v>0.22</v>
+      </c>
+      <c r="M55">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="56" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L56">
+        <v>0.19</v>
+      </c>
+      <c r="M56">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="57" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L57">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="M57">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="58" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L58">
+        <v>0.12</v>
+      </c>
+      <c r="M58">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="59" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L59">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="M59">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="60" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L60">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="M60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="L61">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5851,30 +6074,30 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <f>A2*8</f>
-        <v>8</v>
+        <f>A2*7</f>
+        <v>7</v>
       </c>
       <c r="C2">
-        <v>8.26</v>
+        <v>7.1</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:D6" si="0">B2-C2</f>
-        <v>-0.25999999999999979</v>
+        <v>-9.9999999999999645E-2</v>
       </c>
       <c r="E2" s="1">
         <f>D2/B2</f>
-        <v>-3.2499999999999973E-2</v>
+        <v>-1.4285714285714235E-2</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>7.07</v>
       </c>
       <c r="G2">
         <f>F2-B2</f>
-        <v>-8</v>
+        <v>7.0000000000000284E-2</v>
       </c>
       <c r="H2" s="1">
         <f>G2/B2</f>
-        <v>-1</v>
+        <v>1.000000000000004E-2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
@@ -5882,30 +6105,30 @@
         <v>1.5</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B6" si="1">A3*8</f>
-        <v>12</v>
+        <f t="shared" ref="B3:B6" si="1">A3*7</f>
+        <v>10.5</v>
       </c>
       <c r="C3">
-        <v>12.1</v>
+        <v>10.509</v>
       </c>
       <c r="D3">
         <f t="shared" si="0"/>
-        <v>-9.9999999999999645E-2</v>
+        <v>-9.0000000000003411E-3</v>
       </c>
       <c r="E3" s="1">
         <f t="shared" ref="E3:E6" si="2">D3/B3</f>
-        <v>-8.3333333333333037E-3</v>
+        <v>-8.5714285714288962E-4</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>10.507999999999999</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G6" si="3">F3-B3</f>
-        <v>-12</v>
+        <v>7.9999999999991189E-3</v>
       </c>
       <c r="H3" s="1">
         <f t="shared" ref="H3:H6" si="4">G3/B3</f>
-        <v>-1</v>
+        <v>7.6190476190467801E-4</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
@@ -5914,29 +6137,29 @@
       </c>
       <c r="B4">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4">
-        <v>16.02</v>
+        <v>13.846</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>-1.9999999999999574E-2</v>
+        <v>0.15399999999999991</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" si="2"/>
-        <v>-1.2499999999999734E-3</v>
+        <v>1.0999999999999994E-2</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>14.012</v>
       </c>
       <c r="G4">
         <f t="shared" si="3"/>
-        <v>-16</v>
+        <v>1.2000000000000455E-2</v>
       </c>
       <c r="H4" s="1">
         <f t="shared" si="4"/>
-        <v>-1</v>
+        <v>8.5714285714288962E-4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
@@ -5945,29 +6168,29 @@
       </c>
       <c r="B5">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="C5">
-        <v>19.93</v>
+        <v>17.396000000000001</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>7.0000000000000284E-2</v>
+        <v>0.1039999999999992</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" si="2"/>
-        <v>3.5000000000000144E-3</v>
+        <v>5.942857142857097E-3</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>17.516999999999999</v>
       </c>
       <c r="G5">
         <f t="shared" si="3"/>
-        <v>-20</v>
+        <v>1.699999999999946E-2</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="4"/>
-        <v>-1</v>
+        <v>9.7142857142854054E-4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
@@ -5976,29 +6199,29 @@
       </c>
       <c r="B6">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C6">
-        <v>23.92</v>
+        <v>20.661999999999999</v>
       </c>
       <c r="D6">
         <f t="shared" si="0"/>
-        <v>7.9999999999998295E-2</v>
+        <v>0.33800000000000097</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="2"/>
-        <v>3.3333333333332624E-3</v>
+        <v>1.6095238095238142E-2</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>21.021999999999998</v>
       </c>
       <c r="G6">
         <f t="shared" si="3"/>
-        <v>-24</v>
+        <v>2.1999999999998465E-2</v>
       </c>
       <c r="H6" s="1">
         <f t="shared" si="4"/>
-        <v>-1</v>
+        <v>1.0476190476189746E-3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
@@ -6007,19 +6230,19 @@
       </c>
       <c r="D8">
         <f>AVERAGE(D2:D6)</f>
-        <v>-4.6000000000000082E-2</v>
+        <v>9.7400000000000014E-2</v>
       </c>
       <c r="E8" s="2">
         <f>AVERAGE(E2:E6)</f>
-        <v>-7.0499999999999938E-3</v>
+        <v>3.5790476190476219E-3</v>
       </c>
       <c r="G8">
         <f>AVERAGE(G2:G6)</f>
-        <v>-16</v>
+        <v>2.5799999999999556E-2</v>
       </c>
       <c r="H8" s="2">
         <f>AVERAGE(H2:H6)</f>
-        <v>-1</v>
+        <v>2.7276190476190243E-3</v>
       </c>
     </row>
   </sheetData>
@@ -6069,30 +6292,30 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <f>A2*9</f>
-        <v>9</v>
+        <f t="shared" ref="B2:B5" si="0">A2*7/2</f>
+        <v>3.5</v>
       </c>
       <c r="C2">
-        <v>9.0399999999999991</v>
+        <v>3.621</v>
       </c>
       <c r="D2">
-        <f t="shared" ref="D2:D6" si="0">B2-C2</f>
-        <v>-3.9999999999999147E-2</v>
+        <f t="shared" ref="D2:D6" si="1">B2-C2</f>
+        <v>-0.121</v>
       </c>
       <c r="E2" s="1">
         <f>D2/B2</f>
-        <v>-4.4444444444443499E-3</v>
+        <v>-3.4571428571428572E-2</v>
       </c>
       <c r="F2">
-        <v>9.07</v>
+        <v>3.5339999999999998</v>
       </c>
       <c r="G2">
         <f>F2-B2</f>
-        <v>7.0000000000000284E-2</v>
+        <v>3.3999999999999808E-2</v>
       </c>
       <c r="H2" s="1">
         <f>G2/B2</f>
-        <v>7.7777777777778096E-3</v>
+        <v>9.7142857142856597E-3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
@@ -6100,30 +6323,30 @@
         <v>1.5</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B6" si="1">A3*9</f>
-        <v>13.5</v>
+        <f t="shared" si="0"/>
+        <v>5.25</v>
       </c>
       <c r="C3">
-        <v>13.52</v>
+        <v>5.3609999999999998</v>
       </c>
       <c r="D3">
-        <f t="shared" si="0"/>
-        <v>-1.9999999999999574E-2</v>
+        <f t="shared" si="1"/>
+        <v>-0.11099999999999977</v>
       </c>
       <c r="E3" s="1">
         <f t="shared" ref="E3:E6" si="2">D3/B3</f>
-        <v>-1.48148148148145E-3</v>
+        <v>-2.1142857142857099E-2</v>
       </c>
       <c r="F3">
-        <v>13.57</v>
+        <v>5.29</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G6" si="3">F3-B3</f>
-        <v>7.0000000000000284E-2</v>
+        <v>4.0000000000000036E-2</v>
       </c>
       <c r="H3" s="1">
         <f t="shared" ref="H3:H6" si="4">G3/B3</f>
-        <v>5.1851851851852059E-3</v>
+        <v>7.619047619047626E-3</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
@@ -6131,30 +6354,30 @@
         <v>2</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>7.0650000000000004</v>
+      </c>
+      <c r="D4">
         <f t="shared" si="1"/>
-        <v>18</v>
-      </c>
-      <c r="C4">
-        <v>17.79</v>
-      </c>
-      <c r="D4">
-        <f t="shared" si="0"/>
-        <v>0.21000000000000085</v>
+        <v>-6.5000000000000391E-2</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" si="2"/>
-        <v>1.1666666666666714E-2</v>
+        <v>-9.2857142857143415E-3</v>
       </c>
       <c r="F4">
-        <v>18.07</v>
+        <v>7.0990000000000002</v>
       </c>
       <c r="G4">
         <f t="shared" si="3"/>
-        <v>7.0000000000000284E-2</v>
+        <v>9.9000000000000199E-2</v>
       </c>
       <c r="H4" s="1">
         <f t="shared" si="4"/>
-        <v>3.8888888888889048E-3</v>
+        <v>1.4142857142857171E-2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
@@ -6162,30 +6385,30 @@
         <v>2.5</v>
       </c>
       <c r="B5">
+        <f t="shared" si="0"/>
+        <v>8.75</v>
+      </c>
+      <c r="C5">
+        <v>8.7690000000000001</v>
+      </c>
+      <c r="D5">
         <f t="shared" si="1"/>
-        <v>22.5</v>
-      </c>
-      <c r="C5">
-        <v>22.21</v>
-      </c>
-      <c r="D5">
-        <f t="shared" si="0"/>
-        <v>0.28999999999999915</v>
+        <v>-1.9000000000000128E-2</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" si="2"/>
-        <v>1.2888888888888851E-2</v>
+        <v>-2.1714285714285859E-3</v>
       </c>
       <c r="F5">
-        <v>22.35</v>
+        <v>8.7560000000000002</v>
       </c>
       <c r="G5">
         <f t="shared" si="3"/>
-        <v>-0.14999999999999858</v>
+        <v>6.0000000000002274E-3</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="4"/>
-        <v>-6.6666666666666038E-3</v>
+        <v>6.8571428571431172E-4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
@@ -6193,30 +6416,30 @@
         <v>3</v>
       </c>
       <c r="B6">
+        <f>A6*7/2</f>
+        <v>10.5</v>
+      </c>
+      <c r="C6">
+        <v>10.36</v>
+      </c>
+      <c r="D6">
         <f t="shared" si="1"/>
-        <v>27</v>
-      </c>
-      <c r="C6">
-        <v>26.76</v>
-      </c>
-      <c r="D6">
-        <f t="shared" si="0"/>
-        <v>0.23999999999999844</v>
+        <v>0.14000000000000057</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="2"/>
-        <v>8.8888888888888316E-3</v>
+        <v>1.3333333333333388E-2</v>
       </c>
       <c r="F6">
-        <v>27</v>
+        <v>10.56</v>
       </c>
       <c r="G6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>6.0000000000000497E-2</v>
       </c>
       <c r="H6" s="1">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>5.714285714285762E-3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
@@ -6225,19 +6448,19 @@
       </c>
       <c r="D8">
         <f>AVERAGE(D2:D6)</f>
-        <v>0.13599999999999995</v>
+        <v>-3.519999999999994E-2</v>
       </c>
       <c r="E8" s="2">
         <f>AVERAGE(E2:E6)</f>
-        <v>5.5037037037037198E-3</v>
+        <v>-1.0767619047619043E-2</v>
       </c>
       <c r="G8">
         <f>AVERAGE(G2:G6)</f>
-        <v>1.2000000000000455E-2</v>
+        <v>4.7800000000000155E-2</v>
       </c>
       <c r="H8" s="2">
         <f>AVERAGE(H2:H6)</f>
-        <v>2.0370370370370633E-3</v>
+        <v>7.5752380952381054E-3</v>
       </c>
     </row>
   </sheetData>
@@ -6291,26 +6514,26 @@
         <v>10</v>
       </c>
       <c r="C2">
-        <v>10.46</v>
+        <v>10.29</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:D6" si="0">B2-C2</f>
-        <v>-0.46000000000000085</v>
+        <v>-0.28999999999999915</v>
       </c>
       <c r="E2" s="1">
         <f>D2/B2</f>
-        <v>-4.6000000000000082E-2</v>
+        <v>-2.8999999999999915E-2</v>
       </c>
       <c r="F2">
-        <v>9.9600000000000009</v>
+        <v>9.99</v>
       </c>
       <c r="G2">
         <f>F2-B2</f>
-        <v>-3.9999999999999147E-2</v>
+        <v>-9.9999999999997868E-3</v>
       </c>
       <c r="H2" s="1">
         <f>G2/B2</f>
-        <v>-3.9999999999999151E-3</v>
+        <v>-9.9999999999997877E-4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
@@ -6322,26 +6545,26 @@
         <v>15</v>
       </c>
       <c r="C3">
-        <v>15.37</v>
+        <v>14.98</v>
       </c>
       <c r="D3">
         <f t="shared" si="0"/>
-        <v>-0.36999999999999922</v>
+        <v>1.9999999999999574E-2</v>
       </c>
       <c r="E3" s="1">
         <f t="shared" ref="E3:E6" si="2">D3/B3</f>
-        <v>-2.4666666666666615E-2</v>
+        <v>1.3333333333333049E-3</v>
       </c>
       <c r="F3">
-        <v>15.02</v>
+        <v>15.01</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G6" si="3">F3-B3</f>
-        <v>1.9999999999999574E-2</v>
+        <v>9.9999999999997868E-3</v>
       </c>
       <c r="H3" s="1">
         <f t="shared" ref="H3:H6" si="4">G3/B3</f>
-        <v>1.3333333333333049E-3</v>
+        <v>6.6666666666665244E-4</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
@@ -6353,26 +6576,26 @@
         <v>20</v>
       </c>
       <c r="C4">
-        <v>20.36</v>
+        <v>20.09</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>-0.35999999999999943</v>
+        <v>-8.9999999999999858E-2</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" si="2"/>
-        <v>-1.7999999999999971E-2</v>
+        <v>-4.4999999999999927E-3</v>
       </c>
       <c r="F4">
-        <v>19.97</v>
+        <v>20.02</v>
       </c>
       <c r="G4">
         <f t="shared" si="3"/>
-        <v>-3.0000000000001137E-2</v>
+        <v>1.9999999999999574E-2</v>
       </c>
       <c r="H4" s="1">
         <f t="shared" si="4"/>
-        <v>-1.5000000000000568E-3</v>
+        <v>9.9999999999997877E-4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
@@ -6384,26 +6607,26 @@
         <v>25</v>
       </c>
       <c r="C5">
-        <v>25.41</v>
+        <v>24.85</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>-0.41000000000000014</v>
+        <v>0.14999999999999858</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" si="2"/>
-        <v>-1.6400000000000005E-2</v>
+        <v>5.9999999999999429E-3</v>
       </c>
       <c r="F5">
-        <v>25.03</v>
+        <v>24.98</v>
       </c>
       <c r="G5">
         <f t="shared" si="3"/>
-        <v>3.0000000000001137E-2</v>
+        <v>-1.9999999999999574E-2</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="4"/>
-        <v>1.2000000000000454E-3</v>
+        <v>-7.9999999999998291E-4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
@@ -6415,26 +6638,26 @@
         <v>30</v>
       </c>
       <c r="C6">
-        <v>30.25</v>
+        <v>30.1</v>
       </c>
       <c r="D6">
         <f t="shared" si="0"/>
-        <v>-0.25</v>
+        <v>-0.10000000000000142</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="2"/>
-        <v>-8.3333333333333332E-3</v>
+        <v>-3.3333333333333808E-3</v>
       </c>
       <c r="F6">
-        <v>30.04</v>
+        <v>29.93</v>
       </c>
       <c r="G6">
         <f t="shared" si="3"/>
-        <v>3.9999999999999147E-2</v>
+        <v>-7.0000000000000284E-2</v>
       </c>
       <c r="H6" s="1">
         <f t="shared" si="4"/>
-        <v>1.3333333333333049E-3</v>
+        <v>-2.3333333333333426E-3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
@@ -6443,19 +6666,19 @@
       </c>
       <c r="D8">
         <f>AVERAGE(D2:D6)</f>
-        <v>-0.36999999999999994</v>
+        <v>-6.2000000000000458E-2</v>
       </c>
       <c r="E8" s="2">
         <f>AVERAGE(E2:E6)</f>
-        <v>-2.2679999999999999E-2</v>
+        <v>-5.9000000000000077E-3</v>
       </c>
       <c r="G8">
         <f>AVERAGE(G2:G6)</f>
-        <v>3.9999999999999151E-3</v>
+        <v>-1.4000000000000058E-2</v>
       </c>
       <c r="H8" s="2">
         <f>AVERAGE(H2:H6)</f>
-        <v>-3.2666666666666337E-4</v>
+        <v>-4.9333333333333456E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>